<commit_message>
Make change chunk to graph and make project more practicle
</commit_message>
<xml_diff>
--- a/data/sbc_test_result.xlsx
+++ b/data/sbc_test_result.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="30">
   <si>
     <t>SN</t>
   </si>
@@ -64,7 +64,7 @@
     <t>Yes. $300 for prescription drug coverage and $300 for occupational therapy services.</t>
   </si>
   <si>
-    <t>Yes. There are specific deductibles for pregnancy and childbirth ($500), chronic disease management ($800), and emergency care ($700).</t>
+    <t>Yes. There are other deductibles for specific services. The Pregnancy &amp; Childbirth Scenario has a deductible of $500. The Chronic Disease Management Scenario has a deductible of $800. The Emergency Care Scenario has a deductible of $700. Additionally, there is a $300 deductible for prescription drug coverage and a $300 deductible for occupational therapy services. You must pay all of the costs for these services up to the specific deductible amount before the plan begins to pay for them.</t>
   </si>
   <si>
     <t xml:space="preserve">What is the out-of-pocket limit for this plan? </t>
@@ -73,7 +73,7 @@
     <t>For network providers $2,500 individual / $5,000 family; for out of-network providers $4,000 individual / $8,000 family</t>
   </si>
   <si>
-    <t>The out-of-pocket limit for this plan is $2,500 for individuals and $5,000 for families for network providers, and $4,000 for individuals and $8,000 for families for out-of-network providers.</t>
+    <t>The out-of-pocket limit for this plan is $2,500 for an individual and $5,000 for a family when using network providers, and $4,000 for an individual and $8,000 for a family when using out-of-network providers.</t>
   </si>
   <si>
     <t>What is not included in the out-of-pocket limit?</t>
@@ -82,7 +82,7 @@
     <t>Copayments for certain services, premiums, balance-billed charges, and health care this plan doesn’t cover.</t>
   </si>
   <si>
-    <t>The out-of-pocket limit does not include copayments for certain services, premiums, balance-billed charges, and health care this plan doesn’t cover.</t>
+    <t>The out-of-pocket limit does not include Copayments for certain services, premiums, balance-billed charges, and health care this plan doesn’t cover.</t>
   </si>
   <si>
     <t xml:space="preserve">Will you pay less if you use a network provider? </t>
@@ -91,28 +91,19 @@
     <t>Yes. See www.[insert].com or call 1-800-[insert] for a list of networkproviders.</t>
   </si>
   <si>
-    <t>Yes. Using a network provider typically results in lower costs.</t>
+    <t>Yes. Using a network provider will generally result in lower costs. For a list of network providers, see www.[insert].com or call 1-800-[insert].</t>
   </si>
   <si>
     <t>What is the copay for a primary care visit?</t>
   </si>
   <si>
-    <t>The copay for a primary care visit is $35.</t>
-  </si>
-  <si>
     <t>What is the copay for a diagnostic test (x-ray, blood work)?</t>
   </si>
   <si>
-    <t>The copay for a diagnostic test (x-ray, blood work) is $10 per test.</t>
-  </si>
-  <si>
     <t>What is the copay for imaging tests like MRI?</t>
   </si>
   <si>
     <t>What is the coinsurance for non-preferred brand drugs (Tier 3) in-network?</t>
-  </si>
-  <si>
-    <t>The coinsurance for non-preferred brand drugs (Tier 3) in-network is 40%.</t>
   </si>
 </sst>
 </file>
@@ -547,16 +538,16 @@
         <v>11</v>
       </c>
       <c r="E2" s="4">
-        <v>2909</v>
+        <v>3416</v>
       </c>
       <c r="F2" s="4">
         <v>66</v>
       </c>
       <c r="G2" s="4">
-        <v>2975</v>
+        <v>3482</v>
       </c>
       <c r="H2" s="5">
-        <v>8.07</v>
+        <v>6.78</v>
       </c>
       <c r="I2" s="4">
         <v>0</v>
@@ -576,16 +567,16 @@
         <v>13</v>
       </c>
       <c r="E3" s="4">
-        <v>2943</v>
+        <v>3445</v>
       </c>
       <c r="F3" s="4">
         <v>92</v>
       </c>
       <c r="G3" s="4">
-        <v>3035</v>
+        <v>3537</v>
       </c>
       <c r="H3" s="5">
-        <v>6.54</v>
+        <v>6.14</v>
       </c>
       <c r="I3" s="4">
         <v>1</v>
@@ -605,19 +596,19 @@
         <v>16</v>
       </c>
       <c r="E4" s="4">
-        <v>3424</v>
+        <v>4424</v>
       </c>
       <c r="F4" s="4">
-        <v>128</v>
+        <v>209</v>
       </c>
       <c r="G4" s="4">
-        <v>3552</v>
+        <v>4633</v>
       </c>
       <c r="H4" s="5">
-        <v>8.57</v>
+        <v>11.72</v>
       </c>
       <c r="I4" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
@@ -634,16 +625,16 @@
         <v>19</v>
       </c>
       <c r="E5" s="4">
-        <v>2967</v>
+        <v>3469</v>
       </c>
       <c r="F5" s="4">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="G5" s="4">
-        <v>3074</v>
+        <v>3588</v>
       </c>
       <c r="H5" s="5">
-        <v>6.94</v>
+        <v>6.45</v>
       </c>
       <c r="I5" s="4">
         <v>1</v>
@@ -663,16 +654,16 @@
         <v>22</v>
       </c>
       <c r="E6" s="4">
-        <v>2949</v>
+        <v>3451</v>
       </c>
       <c r="F6" s="4">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="G6" s="4">
-        <v>3034</v>
+        <v>3542</v>
       </c>
       <c r="H6" s="5">
-        <v>6.46</v>
+        <v>5.54</v>
       </c>
       <c r="I6" s="4">
         <v>1</v>
@@ -692,16 +683,16 @@
         <v>25</v>
       </c>
       <c r="E7" s="4">
-        <v>2952</v>
+        <v>3454</v>
       </c>
       <c r="F7" s="4">
-        <v>89</v>
+        <v>114</v>
       </c>
       <c r="G7" s="4">
-        <v>3041</v>
+        <v>3568</v>
       </c>
       <c r="H7" s="5">
-        <v>7.44</v>
+        <v>5.91</v>
       </c>
       <c r="I7" s="4">
         <v>1</v>
@@ -718,22 +709,22 @@
         <v>35</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="E8" s="4">
-        <v>3528</v>
+        <v>3899</v>
       </c>
       <c r="F8" s="4">
-        <v>223</v>
+        <v>313</v>
       </c>
       <c r="G8" s="4">
-        <v>3751</v>
+        <v>4212</v>
       </c>
       <c r="H8" s="5">
-        <v>12.45</v>
+        <v>13.82</v>
       </c>
       <c r="I8" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
@@ -741,28 +732,28 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C9" s="4">
         <v>10</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="E9" s="4">
-        <v>3491</v>
+        <v>4002</v>
       </c>
       <c r="F9" s="4">
-        <v>231</v>
+        <v>313</v>
       </c>
       <c r="G9" s="4">
-        <v>3722</v>
+        <v>4315</v>
       </c>
       <c r="H9" s="5">
-        <v>10.91</v>
+        <v>11.56</v>
       </c>
       <c r="I9" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
@@ -770,7 +761,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C10" s="4">
         <v>50</v>
@@ -779,16 +770,16 @@
         <v>11</v>
       </c>
       <c r="E10" s="4">
-        <v>2904</v>
+        <v>3406</v>
       </c>
       <c r="F10" s="4">
-        <v>218</v>
+        <v>313</v>
       </c>
       <c r="G10" s="4">
-        <v>3122</v>
+        <v>3719</v>
       </c>
       <c r="H10" s="5">
-        <v>10.17</v>
+        <v>10.95</v>
       </c>
       <c r="I10" s="4">
         <v>0</v>
@@ -799,28 +790,28 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C11" s="5">
         <v>0.4</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="E11" s="4">
-        <v>3356</v>
+        <v>3422</v>
       </c>
       <c r="F11" s="4">
-        <v>237</v>
+        <v>318</v>
       </c>
       <c r="G11" s="4">
-        <v>3593</v>
+        <v>3740</v>
       </c>
       <c r="H11" s="5">
-        <v>10.99</v>
+        <v>11.51</v>
       </c>
       <c r="I11" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>